<commit_message>
Recolorer les en-tetes de niveau 1 des plans imbriques en orange
Demande explicite : niveau 1 (famille/module/type) en orange, gras -
niveaux 2/3 inchanges (deja valides). Nouvelle variable dediee
level1Orange (RGB 211,84,0) plutot qu'un renommage global du violet
Ankrr existant, qui servait aussi de couleur de texte-accent ailleurs
et de couleur de serie sur les 3 graphiques de "Vue d'ensemble" - ces
usages restent inchanges.

Applique sur les 4 feuilles a plan imbrique : "Jobs et cycles"/"Jobs
par type de traitement" (dossier d'exploitation, theme sombre) et
"Catalogue des operations"/"Operations par type traitement" (tableau
de bord, theme clair).

Verifie : couleurs relues via COM sur les 2 classeurs (orange confirme
sur toutes les lignes de niveau 1, niveaux 2/3 inchanges), export PDF
reel sur une feuille de chaque theme - orange lisible et coherent sur
fond sombre et fond clair, texte blanc gras toujours contraste.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DOSSIER_EXPLOITATION_QUOTIDIEN.xlsx
+++ b/docs/DOSSIER_EXPLOITATION_QUOTIDIEN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP PROBOOK\Documents\ECF\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{55A0B0EC-1611-434F-BF11-AC921E0F3A03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3768F71B-70F7-4774-9977-CF391CACC44E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5604" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{F5A6BB3A-89A6-4021-B029-5C8BC4A1C3B8}"/>
+    <workbookView xWindow="732" yWindow="732" windowWidth="17280" windowHeight="8880" xr2:uid="{419C3045-35AF-4F04-A9CB-D6E2301278CA}"/>
   </bookViews>
   <sheets>
     <sheet name="Mode d'emploi" sheetId="1" r:id="rId1"/>
@@ -1666,7 +1666,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF9669EB"/>
+        <fgColor rgb="FFD35400"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2063,7 +2063,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC0BF25B-CC6D-4354-8C36-4A1631E81F68}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32E09FAD-AEFF-46A6-9E0A-A10B5D150AFE}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2318,7 +2318,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{445F5AAB-F7E3-4E1A-B00F-F65CE4CD40E4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6624E96-2FB4-4E48-845A-6860D0FB2F3A}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2432,7 +2432,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C79BEE6B-D6FC-435E-AC94-A0B33E844ABC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD676AB5-3BD1-4B39-9235-68C643B6E648}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="1"/>
@@ -4169,7 +4169,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:J3" xr:uid="{C79BEE6B-D6FC-435E-AC94-A0B33E844ABC}"/>
+  <autoFilter ref="A3:J3" xr:uid="{BD676AB5-3BD1-4B39-9235-68C643B6E648}"/>
   <mergeCells count="44">
     <mergeCell ref="A76:J76"/>
     <mergeCell ref="A78:J78"/>
@@ -4226,7 +4226,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BC87A21-33BD-4679-99E2-8BD7169C6A34}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F3EA0A5-0216-4FD8-A081-439BA5DD2F0A}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="1"/>
@@ -5963,7 +5963,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:J3" xr:uid="{5BC87A21-33BD-4679-99E2-8BD7169C6A34}"/>
+  <autoFilter ref="A3:J3" xr:uid="{2F3EA0A5-0216-4FD8-A081-439BA5DD2F0A}"/>
   <mergeCells count="44">
     <mergeCell ref="A77:J77"/>
     <mergeCell ref="A78:J78"/>
@@ -6020,7 +6020,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31C905C3-0765-4BAE-A530-E9FF0A9CFE10}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46BF38C8-876A-4552-8523-55F5659BFB65}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -6319,7 +6319,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G4" xr:uid="{31C905C3-0765-4BAE-A530-E9FF0A9CFE10}"/>
+  <autoFilter ref="A4:G4" xr:uid="{46BF38C8-876A-4552-8523-55F5659BFB65}"/>
   <mergeCells count="2">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
@@ -6334,7 +6334,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8959E6DB-B7C6-44D9-BAA3-F78703DCC6B0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87F88ED2-2D74-4345-A588-4083D685D007}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -6504,7 +6504,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{063B856D-FD6C-46FC-A0CA-5BA267856166}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51AFEDCC-C966-48B3-AEAC-B51127CB52F3}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>

</xml_diff>